<commit_message>
fix: validar tasas y fórmulas del IT-1
</commit_message>
<xml_diff>
--- a/frontend/templates/IT-1-DGII-2020.xlsx
+++ b/frontend/templates/IT-1-DGII-2020.xlsx
@@ -4264,9 +4264,9 @@
       <c r="V5" s="11"/>
       <c r="W5" s="11"/>
       <c r="X5" s="12"/>
-      <c r="Z5" s="2" t="e">
-        <f aca="false">+IF(#REF!="",1,2)</f>
-        <v>#REF!</v>
+      <c r="Z5" s="2">
+        <f aca="false">IF('IT-1'!V14=0,1,2)</f>
+        <v>1</v>
       </c>
       <c r="AN5" s="2"/>
       <c r="AO5" s="2"/>

</xml_diff>